<commit_message>
fix(ble): send one daily settlement summary
</commit_message>
<xml_diff>
--- a/docs/Kirole_BLE协议命令字节表_专注重连协议更新_Ver_1_3_1.xlsx
+++ b/docs/Kirole_BLE协议命令字节表_专注重连协议更新_Ver_1_3_1.xlsx
@@ -11503,7 +11503,7 @@
       </c>
       <c r="F20" s="48" t="inlineStr">
         <is>
-          <t>每日总结页·概况点评（v2.6.0）；空串=尚未生成</t>
+          <t>每日总结页唯一气泡的完整文案：先总结今天；明天有日历安排时带最早一项，若无日历安排则带优先级最高的未完成明日任务，并给出鼓励；两者皆无时用金句收尾</t>
         </is>
       </c>
     </row>
@@ -11533,7 +11533,7 @@
       </c>
       <c r="F21" s="47" t="inlineStr">
         <is>
-          <t>每日总结页·金句/明日鼓励（v2.6.0）；DayPack 当前最后一个字段</t>
+          <t>保留字段；App 当前恒发长度 0，固件必须消费该长度字节但不得渲染；DayPack 最后一个字段</t>
         </is>
       </c>
     </row>

</xml_diff>